<commit_message>
SII Review Tool: Alternative Extrapolation with VA.
</commit_message>
<xml_diff>
--- a/inputs.xlsx
+++ b/inputs.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\d-fine\Projects\SII Review Tool\Tool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\d-fine\Projects\SII Review Tool\SII Review Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{827DD131-AA09-4B8F-B211-00446D76A3EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B45521-67E3-40F5-A969-625CB904174A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
SII Review Tool: Refactoring of MarketData and ExtrapolationAlt. Implementation of ExtrapolationSW.
</commit_message>
<xml_diff>
--- a/inputs.xlsx
+++ b/inputs.xlsx
@@ -8,13 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\d-fine\Projects\SII Review Tool\SII Review Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B45521-67E3-40F5-A969-625CB904174A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF5DC7AB-ECA3-4506-8C82-1270AE563070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="rates" sheetId="1" r:id="rId1"/>
+    <sheet name="rates_alt" sheetId="1" r:id="rId1"/>
+    <sheet name="rates_sw" sheetId="2" r:id="rId2"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId3"/>
+  </externalReferences>
+  <definedNames>
+    <definedName name="BBDATA">OFFSET('[1]INPUT DATA'!$C$8,0,0,'[1]INPUT DATA'!$A$6,50)</definedName>
+    <definedName name="CalcDate" localSheetId="1">rates_sw!$D$4</definedName>
+    <definedName name="DateList">OFFSET('[1]INPUT DATA'!$B$8,0,0,'[1]INPUT DATA'!$A$6,1)</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="4">
   <si>
     <t>Tenor</t>
   </si>
@@ -54,13 +63,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -80,14 +95,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 3" xfId="1" xr:uid="{2351E727-7914-4128-83BF-CE6273F2D9EE}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -100,6 +117,46 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Read Me "/>
+      <sheetName val="Smith-Wilson RFR"/>
+      <sheetName val="Graphs"/>
+      <sheetName val="INPUT DATA"/>
+      <sheetName val="LOG"/>
+      <sheetName val="Sheet1"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3">
+        <row r="6">
+          <cell r="A6">
+            <v>50</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="B8">
+            <v>41640</v>
+          </cell>
+          <cell r="C8">
+            <v>1.8644559400154886E-2</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2492,4 +2549,581 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA0E8BDC-F229-420E-9A56-65EC6A90BF84}">
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1:C51"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="7.6640625" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>9.2496718772093669E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1.0589694258098003E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>1.1032270549913577E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>1.1044292518813812E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>1.3788334788232146E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7">
+        <v>1.6944242364738148E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8">
+        <v>1.8429378313447282E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9">
+        <v>1.8642466810056619E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>2.0102347240970622E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11">
+        <v>2.1872288777203999E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>0</v>
+      </c>
+      <c r="B12">
+        <v>11</v>
+      </c>
+      <c r="C12">
+        <v>2.2981233811356312E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13">
+        <v>2.4615215165166154E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>0</v>
+      </c>
+      <c r="B14">
+        <v>13</v>
+      </c>
+      <c r="C14">
+        <v>2.5867811793301054E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>0</v>
+      </c>
+      <c r="B15">
+        <v>14</v>
+      </c>
+      <c r="C15">
+        <v>2.6940024191389973E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>1</v>
+      </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
+      <c r="C16">
+        <v>2.7786457864007751E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>0</v>
+      </c>
+      <c r="B17">
+        <v>16</v>
+      </c>
+      <c r="C17">
+        <v>2.7961998837721332E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>0</v>
+      </c>
+      <c r="B18">
+        <v>17</v>
+      </c>
+      <c r="C18">
+        <v>2.8432307445889947E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>0</v>
+      </c>
+      <c r="B19">
+        <v>18</v>
+      </c>
+      <c r="C19">
+        <v>2.8665104618739178E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>0</v>
+      </c>
+      <c r="B20">
+        <v>19</v>
+      </c>
+      <c r="C20">
+        <v>2.8956926872526014E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>1</v>
+      </c>
+      <c r="B21">
+        <v>20</v>
+      </c>
+      <c r="C21">
+        <v>2.9492299797021254E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>0</v>
+      </c>
+      <c r="B22">
+        <v>21</v>
+      </c>
+      <c r="C22">
+        <v>3.0425194965994863E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>0</v>
+      </c>
+      <c r="B23">
+        <v>22</v>
+      </c>
+      <c r="C23">
+        <v>3.0899262864683863E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>0</v>
+      </c>
+      <c r="B24">
+        <v>23</v>
+      </c>
+      <c r="C24">
+        <v>3.1509179791222114E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>0</v>
+      </c>
+      <c r="B25">
+        <v>24</v>
+      </c>
+      <c r="C25">
+        <v>3.2274458320078969E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>0</v>
+      </c>
+      <c r="B26">
+        <v>25</v>
+      </c>
+      <c r="C26">
+        <v>3.3004411020988313E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>0</v>
+      </c>
+      <c r="B27">
+        <v>26</v>
+      </c>
+      <c r="C27">
+        <v>3.349589889482734E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>0</v>
+      </c>
+      <c r="B28">
+        <v>27</v>
+      </c>
+      <c r="C28">
+        <v>3.3780265686537352E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>0</v>
+      </c>
+      <c r="B29">
+        <v>28</v>
+      </c>
+      <c r="C29">
+        <v>3.4466641415851526E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>0</v>
+      </c>
+      <c r="B30">
+        <v>29</v>
+      </c>
+      <c r="C30">
+        <v>3.4588648213692223E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>0</v>
+      </c>
+      <c r="B31">
+        <v>30</v>
+      </c>
+      <c r="C31">
+        <v>3.4633928585448177E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>0</v>
+      </c>
+      <c r="B32">
+        <v>31</v>
+      </c>
+      <c r="C32">
+        <v>3.4923272597156385E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>0</v>
+      </c>
+      <c r="B33">
+        <v>32</v>
+      </c>
+      <c r="C33">
+        <v>3.541116892193058E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>0</v>
+      </c>
+      <c r="B34">
+        <v>33</v>
+      </c>
+      <c r="C34">
+        <v>3.5713706153336522E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>0</v>
+      </c>
+      <c r="B35">
+        <v>34</v>
+      </c>
+      <c r="C35">
+        <v>3.6297765136776385E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>0</v>
+      </c>
+      <c r="B36">
+        <v>35</v>
+      </c>
+      <c r="C36">
+        <v>3.6464062868989157E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>0</v>
+      </c>
+      <c r="B37">
+        <v>36</v>
+      </c>
+      <c r="C37">
+        <v>3.6835715037200692E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>0</v>
+      </c>
+      <c r="B38">
+        <v>37</v>
+      </c>
+      <c r="C38">
+        <v>3.7061412798874274E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>0</v>
+      </c>
+      <c r="B39">
+        <v>38</v>
+      </c>
+      <c r="C39">
+        <v>3.7461684848288324E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>0</v>
+      </c>
+      <c r="B40">
+        <v>39</v>
+      </c>
+      <c r="C40">
+        <v>3.7774971723381533E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>0</v>
+      </c>
+      <c r="B41">
+        <v>40</v>
+      </c>
+      <c r="C41">
+        <v>3.8056420537358172E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>0</v>
+      </c>
+      <c r="B42">
+        <v>41</v>
+      </c>
+      <c r="C42">
+        <v>3.8489913626744553E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>0</v>
+      </c>
+      <c r="B43">
+        <v>42</v>
+      </c>
+      <c r="C43">
+        <v>3.8828913271326211E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>0</v>
+      </c>
+      <c r="B44">
+        <v>43</v>
+      </c>
+      <c r="C44">
+        <v>3.8915424852211743E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>0</v>
+      </c>
+      <c r="B45">
+        <v>44</v>
+      </c>
+      <c r="C45">
+        <v>3.9224144229902523E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>0</v>
+      </c>
+      <c r="B46">
+        <v>45</v>
+      </c>
+      <c r="C46">
+        <v>3.9421649415220895E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>0</v>
+      </c>
+      <c r="B47">
+        <v>46</v>
+      </c>
+      <c r="C47">
+        <v>3.9495100727106977E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>0</v>
+      </c>
+      <c r="B48">
+        <v>47</v>
+      </c>
+      <c r="C48">
+        <v>3.9679731487326481E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>0</v>
+      </c>
+      <c r="B49">
+        <v>48</v>
+      </c>
+      <c r="C49">
+        <v>3.980159479077483E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>0</v>
+      </c>
+      <c r="B50">
+        <v>49</v>
+      </c>
+      <c r="C50">
+        <v>4.0207915648931766E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>0</v>
+      </c>
+      <c r="B51">
+        <v>50</v>
+      </c>
+      <c r="C51">
+        <v>4.0221039434912016E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
SII Review Tool: Adding input data (spreads).
</commit_message>
<xml_diff>
--- a/inputs.xlsx
+++ b/inputs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\d-fine\Projects\SII Review Tool\SII Review Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4B13B19-C822-4A05-8626-3D1360020ADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5E0D9B-BB3F-49EA-BD09-384FD1A6FB58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -310,7 +310,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -328,24 +328,17 @@
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 3" xfId="1" xr:uid="{2351E727-7914-4128-83BF-CE6273F2D9EE}"/>
     <cellStyle name="Percent 2" xfId="2" xr:uid="{8E3C7290-F3EB-4F4F-810B-1E8706B54683}"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <font>
-        <color theme="0" tint="-4.9958800012207406E-2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9958800012207406E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -3369,7 +3362,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E398A87-82CA-4B50-B75F-313C6B1D2BBE}">
-  <dimension ref="A1:U53"/>
+  <dimension ref="A1:AB54"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" customWidth="1"/>
@@ -3444,85 +3437,65 @@
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2">
-        <f ca="1">RAND()</f>
-        <v>0.32879153275548356</v>
-      </c>
-      <c r="C2">
-        <f t="shared" ref="C2:R3" ca="1" si="0">RAND()</f>
-        <v>0.75329708019983532</v>
-      </c>
-      <c r="D2">
-        <f t="shared" ca="1" si="0"/>
-        <v>3.1900882851673584E-2</v>
-      </c>
-      <c r="E2">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.5561343813362567</v>
-      </c>
-      <c r="F2">
-        <f t="shared" ca="1" si="0"/>
-        <v>3.5156789691012214E-2</v>
-      </c>
-      <c r="G2">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.8057504005152456</v>
-      </c>
-      <c r="H2">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.89500126908120936</v>
-      </c>
-      <c r="I2">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.99169631016811666</v>
-      </c>
-      <c r="J2">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.97791454914364528</v>
-      </c>
-      <c r="K2">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.72527063721151097</v>
-      </c>
-      <c r="L2">
-        <f t="shared" ca="1" si="0"/>
-        <v>2.3263343896113065E-2</v>
-      </c>
-      <c r="M2">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.35624123280862974</v>
-      </c>
-      <c r="N2">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.2883324211136914</v>
-      </c>
-      <c r="O2">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.46798847437607005</v>
-      </c>
-      <c r="P2">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.99718939412882324</v>
-      </c>
-      <c r="Q2">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.11386781022712889</v>
-      </c>
-      <c r="R2">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.96008610376158932</v>
-      </c>
-      <c r="S2">
-        <f t="shared" ref="S2:U3" ca="1" si="1">RAND()</f>
-        <v>0.13331338367232315</v>
-      </c>
-      <c r="T2">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.48135203321645015</v>
-      </c>
-      <c r="U2">
-        <f t="shared" ca="1" si="1"/>
-        <v>5.1857418944855516E-2</v>
+      <c r="B2" s="8">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="C2" s="8">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="D2" s="8">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="E2" s="8">
+        <v>2.5999999999999999E-3</v>
+      </c>
+      <c r="F2" s="8">
+        <v>2.7000000000000001E-3</v>
+      </c>
+      <c r="G2" s="8">
+        <v>2.8E-3</v>
+      </c>
+      <c r="H2" s="8">
+        <v>2.8999999999999998E-3</v>
+      </c>
+      <c r="I2" s="8">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="J2" s="8">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="K2" s="8">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="L2" s="8">
+        <v>3.2499999999999999E-3</v>
+      </c>
+      <c r="M2" s="8">
+        <v>3.3E-3</v>
+      </c>
+      <c r="N2" s="8">
+        <v>3.3500000000000001E-3</v>
+      </c>
+      <c r="O2" s="8">
+        <v>3.3999999999999998E-3</v>
+      </c>
+      <c r="P2" s="8">
+        <v>3.4499999999999999E-3</v>
+      </c>
+      <c r="Q2" s="8">
+        <v>3.5000000000000001E-3</v>
+      </c>
+      <c r="R2" s="8">
+        <v>3.5500000000000002E-3</v>
+      </c>
+      <c r="S2" s="8">
+        <v>3.5999999999999999E-3</v>
+      </c>
+      <c r="T2" s="8">
+        <v>3.65E-3</v>
+      </c>
+      <c r="U2" s="8">
+        <v>3.7000000000000002E-3</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
@@ -3530,84 +3503,64 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <f ca="1">RAND()</f>
-        <v>0.81370766511264525</v>
+        <v>3.8E-3</v>
       </c>
       <c r="C3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.72667639676506335</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="D3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.91791747155625947</v>
+        <v>4.1000000000000003E-3</v>
       </c>
       <c r="E3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.63886731249650153</v>
+        <v>4.1999999999999997E-3</v>
       </c>
       <c r="F3">
-        <f t="shared" ca="1" si="0"/>
-        <v>3.1382472643246007E-2</v>
+        <v>4.3E-3</v>
       </c>
       <c r="G3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.11399323540280337</v>
+        <v>4.4000000000000003E-3</v>
       </c>
       <c r="H3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.34037395865969178</v>
+        <v>4.4999999999999997E-3</v>
       </c>
       <c r="I3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.5821963287956976</v>
+        <v>4.5999999999999999E-3</v>
       </c>
       <c r="J3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.21568181537834574</v>
+        <v>4.7000000000000002E-3</v>
       </c>
       <c r="K3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.18655112329081802</v>
+        <v>4.7999999999999996E-3</v>
       </c>
       <c r="L3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.36796995168392022</v>
+        <v>4.8500000000000001E-3</v>
       </c>
       <c r="M3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.12161721263099567</v>
+        <v>4.8999999999999998E-3</v>
       </c>
       <c r="N3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.3780544620275168</v>
+        <v>4.9500000000000004E-3</v>
       </c>
       <c r="O3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.2360732544573324</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="P3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.49096868533516302</v>
+        <v>5.0499999999999998E-3</v>
       </c>
       <c r="Q3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.12580437303107805</v>
+        <v>5.1000000000000004E-3</v>
       </c>
       <c r="R3">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.33499540482954648</v>
+        <v>5.1500000000000001E-3</v>
       </c>
       <c r="S3">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.34019605613945936</v>
+        <v>5.1999999999999998E-3</v>
       </c>
       <c r="T3">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.31391710111168736</v>
+        <v>5.2500000000000003E-3</v>
       </c>
       <c r="U3">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.23856446983787505</v>
+        <v>5.3E-3</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
@@ -4004,170 +3957,130 @@
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B10">
-        <f t="shared" ref="B10:Q12" ca="1" si="2">RAND()</f>
-        <v>0.28609500297072543</v>
-      </c>
-      <c r="C10">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.19901660806193511</v>
-      </c>
-      <c r="D10">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.6581556714443989</v>
-      </c>
-      <c r="E10">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.81268342660872817</v>
-      </c>
-      <c r="F10">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.46201883193962578</v>
-      </c>
-      <c r="G10">
-        <f t="shared" ca="1" si="2"/>
-        <v>3.1848856190636488E-2</v>
-      </c>
-      <c r="H10">
-        <f t="shared" ca="1" si="2"/>
-        <v>2.5473278331028082E-2</v>
-      </c>
-      <c r="I10">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.54573043006149879</v>
-      </c>
-      <c r="J10">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.87220071738587091</v>
-      </c>
-      <c r="K10">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.14212163255109345</v>
-      </c>
-      <c r="L10">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.11214109566507213</v>
-      </c>
-      <c r="M10">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.14724270150243501</v>
-      </c>
-      <c r="N10">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.40379769916163677</v>
-      </c>
-      <c r="O10">
-        <f t="shared" ca="1" si="2"/>
-        <v>2.7415107181676612E-2</v>
-      </c>
-      <c r="P10">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.80284652653707622</v>
-      </c>
-      <c r="Q10">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.15587525646002254</v>
-      </c>
-      <c r="R10">
-        <f t="shared" ref="R10:U12" ca="1" si="3">RAND()</f>
-        <v>0.27685248365824044</v>
-      </c>
-      <c r="S10">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.45331814262553383</v>
-      </c>
-      <c r="T10">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.70355483833213617</v>
-      </c>
-      <c r="U10">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.14894707603706447</v>
+      <c r="B10" s="8">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="C10" s="8">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="D10" s="8">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="E10" s="8">
+        <v>2.5999999999999999E-3</v>
+      </c>
+      <c r="F10" s="8">
+        <v>2.7000000000000001E-3</v>
+      </c>
+      <c r="G10" s="8">
+        <v>2.8E-3</v>
+      </c>
+      <c r="H10" s="8">
+        <v>2.8999999999999998E-3</v>
+      </c>
+      <c r="I10" s="8">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="J10" s="8">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="K10" s="8">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="L10" s="8">
+        <v>3.2499999999999999E-3</v>
+      </c>
+      <c r="M10" s="8">
+        <v>3.3E-3</v>
+      </c>
+      <c r="N10" s="8">
+        <v>3.3500000000000001E-3</v>
+      </c>
+      <c r="O10" s="8">
+        <v>3.3999999999999998E-3</v>
+      </c>
+      <c r="P10" s="8">
+        <v>3.4499999999999999E-3</v>
+      </c>
+      <c r="Q10" s="8">
+        <v>3.5000000000000001E-3</v>
+      </c>
+      <c r="R10" s="8">
+        <v>3.5500000000000002E-3</v>
+      </c>
+      <c r="S10" s="8">
+        <v>3.5999999999999999E-3</v>
+      </c>
+      <c r="T10" s="8">
+        <v>3.65E-3</v>
+      </c>
+      <c r="U10" s="8">
+        <v>3.7000000000000002E-3</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.90743037639072321</v>
-      </c>
-      <c r="C11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.20574770964166222</v>
-      </c>
-      <c r="D11">
-        <f t="shared" ca="1" si="2"/>
-        <v>9.41107062964186E-2</v>
-      </c>
-      <c r="E11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.99744152501241889</v>
-      </c>
-      <c r="F11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.28064048819033727</v>
-      </c>
-      <c r="G11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.14284376757063966</v>
-      </c>
-      <c r="H11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.98168448579099199</v>
-      </c>
-      <c r="I11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.5311564549363873</v>
-      </c>
-      <c r="J11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.80787625451015044</v>
-      </c>
-      <c r="K11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.65142579502085329</v>
-      </c>
-      <c r="L11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.49402380367600263</v>
-      </c>
-      <c r="M11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.37757229012610438</v>
-      </c>
-      <c r="N11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.55052715449365164</v>
-      </c>
-      <c r="O11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.33462903891059315</v>
-      </c>
-      <c r="P11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.15915411683399305</v>
-      </c>
-      <c r="Q11">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.63819451715410946</v>
-      </c>
-      <c r="R11">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.7233719387003148</v>
-      </c>
-      <c r="S11">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.92659352795056915</v>
-      </c>
-      <c r="T11">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.99945635434475089</v>
-      </c>
-      <c r="U11">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.71338484827790904</v>
+      <c r="B11" s="8">
+        <v>1.20625E-2</v>
+      </c>
+      <c r="C11" s="8">
+        <v>1.2437500000000001E-2</v>
+      </c>
+      <c r="D11" s="8">
+        <v>1.257638888888889E-2</v>
+      </c>
+      <c r="E11" s="8">
+        <v>1.271527777777778E-2</v>
+      </c>
+      <c r="F11" s="8">
+        <v>1.285416666666667E-2</v>
+      </c>
+      <c r="G11" s="8">
+        <v>1.30125E-2</v>
+      </c>
+      <c r="H11" s="8">
+        <v>1.317083333333333E-2</v>
+      </c>
+      <c r="I11" s="8">
+        <v>1.332916666666667E-2</v>
+      </c>
+      <c r="J11" s="8">
+        <v>1.3487499999999999E-2</v>
+      </c>
+      <c r="K11" s="8">
+        <v>1.3645833333333329E-2</v>
+      </c>
+      <c r="L11" s="8">
+        <v>1.3724999999999999E-2</v>
+      </c>
+      <c r="M11" s="8">
+        <v>1.3804166666666669E-2</v>
+      </c>
+      <c r="N11" s="8">
+        <v>1.3883333333333331E-2</v>
+      </c>
+      <c r="O11" s="8">
+        <v>1.3962499999999999E-2</v>
+      </c>
+      <c r="P11" s="8">
+        <v>1.4041666666666669E-2</v>
+      </c>
+      <c r="Q11" s="8">
+        <v>1.4120833333333331E-2</v>
+      </c>
+      <c r="R11" s="8">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="S11" s="8">
+        <v>1.4279166666666669E-2</v>
+      </c>
+      <c r="T11" s="8">
+        <v>1.4358333333333331E-2</v>
+      </c>
+      <c r="U11" s="8">
+        <v>1.4437500000000001E-2</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
@@ -4175,84 +4088,64 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.37006668095109985</v>
+        <v>1E-4</v>
       </c>
       <c r="C12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.79716740534033093</v>
-      </c>
-      <c r="D12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.9751008956793995</v>
-      </c>
-      <c r="E12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.21667400190137687</v>
-      </c>
-      <c r="F12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.81356617706448275</v>
-      </c>
-      <c r="G12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.70700524294876177</v>
-      </c>
-      <c r="H12">
-        <f t="shared" ca="1" si="2"/>
-        <v>5.6252375527537368E-2</v>
-      </c>
-      <c r="I12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.11559376073194094</v>
-      </c>
-      <c r="J12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.47974866185919873</v>
-      </c>
-      <c r="K12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.68442313704009405</v>
-      </c>
-      <c r="L12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.38658597455614929</v>
-      </c>
-      <c r="M12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.12435175477281857</v>
-      </c>
-      <c r="N12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.55063765349971527</v>
-      </c>
-      <c r="O12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.91083068253644817</v>
-      </c>
-      <c r="P12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.73809565011987632</v>
-      </c>
-      <c r="Q12">
-        <f t="shared" ca="1" si="2"/>
-        <v>0.83927346103975875</v>
-      </c>
-      <c r="R12">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.99867259409797349</v>
-      </c>
-      <c r="S12">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.66610466188117845</v>
-      </c>
-      <c r="T12">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.24754690443470928</v>
-      </c>
-      <c r="U12">
-        <f t="shared" ca="1" si="3"/>
-        <v>0.76494809582672518</v>
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="D12" s="8">
+        <v>3.0000000000000003E-4</v>
+      </c>
+      <c r="E12" s="8">
+        <v>4.0000000000000002E-4</v>
+      </c>
+      <c r="F12" s="8">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G12" s="8">
+        <v>6.0000000000000006E-4</v>
+      </c>
+      <c r="H12" s="8">
+        <v>7.000000000000001E-4</v>
+      </c>
+      <c r="I12" s="8">
+        <v>8.0000000000000015E-4</v>
+      </c>
+      <c r="J12" s="8">
+        <v>9.0000000000000019E-4</v>
+      </c>
+      <c r="K12" s="8">
+        <v>1.0000000000000002E-3</v>
+      </c>
+      <c r="L12" s="8">
+        <v>1.1000000000000003E-3</v>
+      </c>
+      <c r="M12" s="8">
+        <v>1.2000000000000003E-3</v>
+      </c>
+      <c r="N12" s="8">
+        <v>1.3000000000000004E-3</v>
+      </c>
+      <c r="O12" s="8">
+        <v>1.4000000000000004E-3</v>
+      </c>
+      <c r="P12" s="8">
+        <v>1.5000000000000005E-3</v>
+      </c>
+      <c r="Q12" s="8">
+        <v>1.6000000000000005E-3</v>
+      </c>
+      <c r="R12" s="8">
+        <v>1.7000000000000006E-3</v>
+      </c>
+      <c r="S12" s="8">
+        <v>1.8000000000000006E-3</v>
+      </c>
+      <c r="T12" s="8">
+        <v>1.9000000000000006E-3</v>
+      </c>
+      <c r="U12" s="8">
+        <v>2.0000000000000005E-3</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
@@ -4455,84 +4348,64 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <f t="shared" ref="B16:Q17" ca="1" si="4">RAND()</f>
-        <v>0.95534972573863486</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="C16">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.23485379432362419</v>
+        <v>2.8999999999999998E-3</v>
       </c>
       <c r="D16">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.84728786303754444</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="E16">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.24321198532369359</v>
+        <v>3.0999999999999999E-3</v>
       </c>
       <c r="F16">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.63006314130900631</v>
+        <v>3.2000000000000002E-3</v>
       </c>
       <c r="G16">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.33350457822470003</v>
+        <v>3.3E-3</v>
       </c>
       <c r="H16">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.16691724858741541</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="I16">
-        <f t="shared" ca="1" si="4"/>
-        <v>7.6089777928422864E-2</v>
+        <v>3.5000000000000001E-3</v>
       </c>
       <c r="J16">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.16623449889883746</v>
+        <v>3.5999999999999999E-3</v>
       </c>
       <c r="K16">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.92462164955751414</v>
+        <v>3.7000000000000002E-3</v>
       </c>
       <c r="L16">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.36691439299406137</v>
+        <v>3.7499999999999999E-3</v>
       </c>
       <c r="M16">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.2504461784666786</v>
+        <v>3.8E-3</v>
       </c>
       <c r="N16">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.21619525436290832</v>
+        <v>3.8500000000000001E-3</v>
       </c>
       <c r="O16">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.59402016706608063</v>
+        <v>3.8999999999999998E-3</v>
       </c>
       <c r="P16">
-        <f t="shared" ca="1" si="4"/>
-        <v>3.0641000245942851E-2</v>
+        <v>3.9500000000000004E-3</v>
       </c>
       <c r="Q16">
-        <f t="shared" ca="1" si="4"/>
-        <v>4.3878823057493355E-2</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="R16">
-        <f t="shared" ref="R16:U17" ca="1" si="5">RAND()</f>
-        <v>0.4293019588990965</v>
+        <v>4.0499999999999998E-3</v>
       </c>
       <c r="S16">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.39789977271852361</v>
+        <v>4.1000000000000003E-3</v>
       </c>
       <c r="T16">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.26191266268874547</v>
+        <v>4.15E-3</v>
       </c>
       <c r="U16">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.53661846874155383</v>
+        <v>4.1999999999999997E-3</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.3">
@@ -4540,84 +4413,64 @@
         <v>19</v>
       </c>
       <c r="B17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.82937223374804547</v>
+        <v>1.14E-2</v>
       </c>
       <c r="C17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.97268840248893473</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="D17">
-        <f t="shared" ca="1" si="4"/>
-        <v>5.1421126556198349E-2</v>
+        <v>1.17E-2</v>
       </c>
       <c r="E17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.58081945667721713</v>
+        <v>1.18E-2</v>
       </c>
       <c r="F17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.83667692845124464</v>
+        <v>1.1900000000000001E-2</v>
       </c>
       <c r="G17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.24482802003561155</v>
+        <v>1.2E-2</v>
       </c>
       <c r="H17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.31548771507875961</v>
+        <v>1.21E-2</v>
       </c>
       <c r="I17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.17734510689275873</v>
+        <v>1.2200000000000001E-2</v>
       </c>
       <c r="J17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.53126211980220506</v>
+        <v>1.23E-2</v>
       </c>
       <c r="K17">
-        <f t="shared" ca="1" si="4"/>
-        <v>4.8545390185432691E-3</v>
+        <v>1.24E-2</v>
       </c>
       <c r="L17">
-        <f t="shared" ca="1" si="4"/>
-        <v>1.2201525619716436E-2</v>
+        <v>1.2449999999999999E-2</v>
       </c>
       <c r="M17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.63129449866576082</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="N17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.2028270507463461</v>
+        <v>1.255E-2</v>
       </c>
       <c r="O17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.28585956529037393</v>
+        <v>1.26E-2</v>
       </c>
       <c r="P17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.25838801163224712</v>
+        <v>1.265E-2</v>
       </c>
       <c r="Q17">
-        <f t="shared" ca="1" si="4"/>
-        <v>0.34673099599185009</v>
+        <v>1.2699999999999999E-2</v>
       </c>
       <c r="R17">
-        <f t="shared" ca="1" si="5"/>
-        <v>8.8205666480333345E-2</v>
+        <v>1.2749999999999999E-2</v>
       </c>
       <c r="S17">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.78341955440427147</v>
+        <v>1.2800000000000001E-2</v>
       </c>
       <c r="T17">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.90934797600586259</v>
+        <v>1.285E-2</v>
       </c>
       <c r="U17">
-        <f t="shared" ca="1" si="5"/>
-        <v>0.69994918789379978</v>
+        <v>1.29E-2</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
@@ -4950,84 +4803,64 @@
         <v>25</v>
       </c>
       <c r="B23">
-        <f t="shared" ref="B23:U23" ca="1" si="6">RAND()</f>
-        <v>0.35885620650313865</v>
+        <v>2.2000000000000001E-3</v>
       </c>
       <c r="C23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.17140996871985015</v>
+        <v>2.3999999999999998E-3</v>
       </c>
       <c r="D23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.79979857821667899</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="E23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.45080413722546753</v>
+        <v>2.5999999999999999E-3</v>
       </c>
       <c r="F23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.28009459146845528</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="G23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.70738348751093039</v>
+        <v>2.8E-3</v>
       </c>
       <c r="H23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.40846745432301867</v>
+        <v>2.8999999999999998E-3</v>
       </c>
       <c r="I23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.23370295854440104</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="J23">
-        <f t="shared" ca="1" si="6"/>
-        <v>6.1671551435345084E-2</v>
+        <v>3.0999999999999999E-3</v>
       </c>
       <c r="K23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.23762893064163748</v>
+        <v>3.2000000000000002E-3</v>
       </c>
       <c r="L23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.64323777939948223</v>
+        <v>3.2499999999999999E-3</v>
       </c>
       <c r="M23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.2229812006428803</v>
+        <v>3.3E-3</v>
       </c>
       <c r="N23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.93698742344403418</v>
+        <v>3.3500000000000001E-3</v>
       </c>
       <c r="O23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.88635402981358402</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="P23">
-        <f t="shared" ca="1" si="6"/>
-        <v>3.8859684963647667E-2</v>
+        <v>3.4499999999999999E-3</v>
       </c>
       <c r="Q23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.70250973248518389</v>
+        <v>3.5000000000000001E-3</v>
       </c>
       <c r="R23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.50839085522241434</v>
+        <v>3.5500000000000002E-3</v>
       </c>
       <c r="S23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.92569618413002097</v>
+        <v>3.5999999999999999E-3</v>
       </c>
       <c r="T23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.20423082076717403</v>
+        <v>3.65E-3</v>
       </c>
       <c r="U23">
-        <f t="shared" ca="1" si="6"/>
-        <v>0.68679146529953694</v>
+        <v>3.7000000000000002E-3</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.3">
@@ -5099,85 +4932,65 @@
       <c r="A25" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B25">
-        <f t="shared" ref="B25:Q26" ca="1" si="7">RAND()</f>
-        <v>6.9596003511846694E-2</v>
-      </c>
-      <c r="C25">
-        <f t="shared" ca="1" si="7"/>
-        <v>4.685267232306678E-2</v>
-      </c>
-      <c r="D25">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.34100079253814419</v>
-      </c>
-      <c r="E25">
-        <f t="shared" ca="1" si="7"/>
-        <v>1.3263426762092023E-2</v>
-      </c>
-      <c r="F25">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.86461897616754946</v>
-      </c>
-      <c r="G25">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.85777521481674168</v>
-      </c>
-      <c r="H25">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.98181061811941095</v>
-      </c>
-      <c r="I25">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.94106864811833668</v>
-      </c>
-      <c r="J25">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.50529669625722451</v>
-      </c>
-      <c r="K25">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.54211918581221841</v>
-      </c>
-      <c r="L25">
-        <f t="shared" ca="1" si="7"/>
-        <v>1.456147084501036E-2</v>
-      </c>
-      <c r="M25">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.41901791669933419</v>
-      </c>
-      <c r="N25">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.14958119485079668</v>
-      </c>
-      <c r="O25">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.15998919757108654</v>
-      </c>
-      <c r="P25">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.97313672829891562</v>
-      </c>
-      <c r="Q25">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.76506546357494587</v>
-      </c>
-      <c r="R25">
-        <f t="shared" ref="R25:U26" ca="1" si="8">RAND()</f>
-        <v>0.59396988012778495</v>
-      </c>
-      <c r="S25">
-        <f t="shared" ca="1" si="8"/>
-        <v>0.39422154094035644</v>
-      </c>
-      <c r="T25">
-        <f t="shared" ca="1" si="8"/>
-        <v>0.90266512462109505</v>
-      </c>
-      <c r="U25">
-        <f t="shared" ca="1" si="8"/>
-        <v>0.2933675523585132</v>
+      <c r="B25" s="8">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="C25" s="8">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="D25" s="8">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="E25" s="8">
+        <v>2.5999999999999999E-3</v>
+      </c>
+      <c r="F25" s="8">
+        <v>2.7000000000000001E-3</v>
+      </c>
+      <c r="G25" s="8">
+        <v>2.8E-3</v>
+      </c>
+      <c r="H25" s="8">
+        <v>2.8999999999999998E-3</v>
+      </c>
+      <c r="I25" s="8">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="J25" s="8">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="K25" s="8">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="L25" s="8">
+        <v>3.2499999999999999E-3</v>
+      </c>
+      <c r="M25" s="8">
+        <v>3.3E-3</v>
+      </c>
+      <c r="N25" s="8">
+        <v>3.3500000000000001E-3</v>
+      </c>
+      <c r="O25" s="8">
+        <v>3.3999999999999998E-3</v>
+      </c>
+      <c r="P25" s="8">
+        <v>3.4499999999999999E-3</v>
+      </c>
+      <c r="Q25" s="8">
+        <v>3.5000000000000001E-3</v>
+      </c>
+      <c r="R25" s="8">
+        <v>3.5500000000000002E-3</v>
+      </c>
+      <c r="S25" s="8">
+        <v>3.5999999999999999E-3</v>
+      </c>
+      <c r="T25" s="8">
+        <v>3.65E-3</v>
+      </c>
+      <c r="U25" s="8">
+        <v>3.7000000000000002E-3</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.3">
@@ -5185,84 +4998,64 @@
         <v>28</v>
       </c>
       <c r="B26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.54383009819791583</v>
+        <v>4.3E-3</v>
       </c>
       <c r="C26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.76735047814612856</v>
+        <v>4.4999999999999997E-3</v>
       </c>
       <c r="D26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.38575361382064821</v>
+        <v>4.5999999999999999E-3</v>
       </c>
       <c r="E26">
-        <f t="shared" ca="1" si="7"/>
-        <v>4.1354739565843235E-2</v>
+        <v>4.7000000000000002E-3</v>
       </c>
       <c r="F26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.94107659743992844</v>
+        <v>4.7999999999999996E-3</v>
       </c>
       <c r="G26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.18952877832710358</v>
+        <v>4.8999999999999998E-3</v>
       </c>
       <c r="H26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.58154519283944051</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="I26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.39973671646996933</v>
+        <v>5.1000000000000004E-3</v>
       </c>
       <c r="J26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.34883583710826815</v>
+        <v>5.1999999999999998E-3</v>
       </c>
       <c r="K26">
-        <f t="shared" ca="1" si="7"/>
-        <v>7.1760913862593423E-2</v>
+        <v>5.3E-3</v>
       </c>
       <c r="L26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.84991410937227296</v>
+        <v>5.3499999999999997E-3</v>
       </c>
       <c r="M26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.33197163905428217</v>
+        <v>5.4000000000000003E-3</v>
       </c>
       <c r="N26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.92415384154134284</v>
+        <v>5.45E-3</v>
       </c>
       <c r="O26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.97908013475248312</v>
+        <v>5.4999999999999997E-3</v>
       </c>
       <c r="P26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.6582481913963828</v>
+        <v>5.5500000000000002E-3</v>
       </c>
       <c r="Q26">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.35771602059493302</v>
+        <v>5.5999999999999999E-3</v>
       </c>
       <c r="R26">
-        <f t="shared" ca="1" si="8"/>
-        <v>0.2028703004594119</v>
+        <v>5.6499999999999996E-3</v>
       </c>
       <c r="S26">
-        <f t="shared" ca="1" si="8"/>
-        <v>0.10831814614954061</v>
+        <v>5.7000000000000002E-3</v>
       </c>
       <c r="T26">
-        <f t="shared" ca="1" si="8"/>
-        <v>0.44242745739253952</v>
+        <v>5.7499999999999999E-3</v>
       </c>
       <c r="U26">
-        <f t="shared" ca="1" si="8"/>
-        <v>0.25850868240146729</v>
+        <v>5.7999999999999996E-3</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.3">
@@ -5334,170 +5127,130 @@
       <c r="A28" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B28">
-        <f t="shared" ref="B28:Q30" ca="1" si="9">RAND()</f>
-        <v>0.95667947026854661</v>
-      </c>
-      <c r="C28">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.19375468102596272</v>
-      </c>
-      <c r="D28">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.89214565312181759</v>
-      </c>
-      <c r="E28">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.85401145105068399</v>
-      </c>
-      <c r="F28">
-        <f t="shared" ca="1" si="9"/>
-        <v>2.2549564321348248E-2</v>
-      </c>
-      <c r="G28">
-        <f t="shared" ca="1" si="9"/>
-        <v>9.2128023342778143E-2</v>
-      </c>
-      <c r="H28">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.50952461353588185</v>
-      </c>
-      <c r="I28">
-        <f t="shared" ca="1" si="9"/>
-        <v>3.8064074340413034E-2</v>
-      </c>
-      <c r="J28">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.56128826541091503</v>
-      </c>
-      <c r="K28">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.86035471067916003</v>
-      </c>
-      <c r="L28">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.29394907435368389</v>
-      </c>
-      <c r="M28">
-        <f t="shared" ca="1" si="9"/>
-        <v>9.901745767207204E-2</v>
-      </c>
-      <c r="N28">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.93498291231659236</v>
-      </c>
-      <c r="O28">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.43854435212754395</v>
-      </c>
-      <c r="P28">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.24087604657069961</v>
-      </c>
-      <c r="Q28">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.70770046217672056</v>
-      </c>
-      <c r="R28">
-        <f t="shared" ref="R28:U30" ca="1" si="10">RAND()</f>
-        <v>0.50292779738814197</v>
-      </c>
-      <c r="S28">
-        <f t="shared" ca="1" si="10"/>
-        <v>0.40028064815595499</v>
-      </c>
-      <c r="T28">
-        <f t="shared" ca="1" si="10"/>
-        <v>0.40241224920296703</v>
-      </c>
-      <c r="U28">
-        <f t="shared" ca="1" si="10"/>
-        <v>0.30119091383404994</v>
+      <c r="B28" s="8">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="C28" s="8">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="D28" s="8">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="E28" s="8">
+        <v>2.5999999999999999E-3</v>
+      </c>
+      <c r="F28" s="8">
+        <v>2.7000000000000001E-3</v>
+      </c>
+      <c r="G28" s="8">
+        <v>2.8E-3</v>
+      </c>
+      <c r="H28" s="8">
+        <v>2.8999999999999998E-3</v>
+      </c>
+      <c r="I28" s="8">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="J28" s="8">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="K28" s="8">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="L28" s="8">
+        <v>3.2499999999999999E-3</v>
+      </c>
+      <c r="M28" s="8">
+        <v>3.3E-3</v>
+      </c>
+      <c r="N28" s="8">
+        <v>3.3500000000000001E-3</v>
+      </c>
+      <c r="O28" s="8">
+        <v>3.3999999999999998E-3</v>
+      </c>
+      <c r="P28" s="8">
+        <v>3.4499999999999999E-3</v>
+      </c>
+      <c r="Q28" s="8">
+        <v>3.5000000000000001E-3</v>
+      </c>
+      <c r="R28" s="8">
+        <v>3.5500000000000002E-3</v>
+      </c>
+      <c r="S28" s="8">
+        <v>3.5999999999999999E-3</v>
+      </c>
+      <c r="T28" s="8">
+        <v>3.65E-3</v>
+      </c>
+      <c r="U28" s="8">
+        <v>3.7000000000000002E-3</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.74374214595681942</v>
-      </c>
-      <c r="C29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.75938590469171752</v>
-      </c>
-      <c r="D29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.93011609701697184</v>
-      </c>
-      <c r="E29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.57712769404625541</v>
-      </c>
-      <c r="F29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.70729979614367455</v>
-      </c>
-      <c r="G29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.94648696384037168</v>
-      </c>
-      <c r="H29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.25588497490452788</v>
-      </c>
-      <c r="I29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.80936653395773595</v>
-      </c>
-      <c r="J29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.40609963021549866</v>
-      </c>
-      <c r="K29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.61234768751097113</v>
-      </c>
-      <c r="L29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.16013121903369898</v>
-      </c>
-      <c r="M29">
-        <f t="shared" ca="1" si="9"/>
-        <v>7.3046434896776424E-2</v>
-      </c>
-      <c r="N29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.30160494982441832</v>
-      </c>
-      <c r="O29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.82040685606814112</v>
-      </c>
-      <c r="P29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.56721943303947464</v>
-      </c>
-      <c r="Q29">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.4628542506292832</v>
-      </c>
-      <c r="R29">
-        <f t="shared" ca="1" si="10"/>
-        <v>0.50934203131306777</v>
-      </c>
-      <c r="S29">
-        <f t="shared" ca="1" si="10"/>
-        <v>0.55580351844379328</v>
-      </c>
-      <c r="T29">
-        <f t="shared" ca="1" si="10"/>
-        <v>0.63727720797744858</v>
-      </c>
-      <c r="U29">
-        <f t="shared" ca="1" si="10"/>
-        <v>0.98301536133943557</v>
+      <c r="B29" s="8">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="C29" s="8">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="D29" s="8">
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="E29" s="8">
+        <v>2.5999999999999999E-3</v>
+      </c>
+      <c r="F29" s="8">
+        <v>2.7000000000000001E-3</v>
+      </c>
+      <c r="G29" s="8">
+        <v>2.8E-3</v>
+      </c>
+      <c r="H29" s="8">
+        <v>2.8999999999999998E-3</v>
+      </c>
+      <c r="I29" s="8">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="J29" s="8">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="K29" s="8">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="L29" s="8">
+        <v>3.2499999999999999E-3</v>
+      </c>
+      <c r="M29" s="8">
+        <v>3.3E-3</v>
+      </c>
+      <c r="N29" s="8">
+        <v>3.3500000000000001E-3</v>
+      </c>
+      <c r="O29" s="8">
+        <v>3.3999999999999998E-3</v>
+      </c>
+      <c r="P29" s="8">
+        <v>3.4499999999999999E-3</v>
+      </c>
+      <c r="Q29" s="8">
+        <v>3.5000000000000001E-3</v>
+      </c>
+      <c r="R29" s="8">
+        <v>3.5500000000000002E-3</v>
+      </c>
+      <c r="S29" s="8">
+        <v>3.5999999999999999E-3</v>
+      </c>
+      <c r="T29" s="8">
+        <v>3.65E-3</v>
+      </c>
+      <c r="U29" s="8">
+        <v>3.7000000000000002E-3</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.3">
@@ -5505,84 +5258,64 @@
         <v>32</v>
       </c>
       <c r="B30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.36148837382099863</v>
+        <v>6.4999999999999997E-3</v>
       </c>
       <c r="C30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.51505299655315262</v>
+        <v>6.7000000000000002E-3</v>
       </c>
       <c r="D30">
-        <f t="shared" ca="1" si="9"/>
-        <v>4.429766998240614E-2</v>
+        <v>6.7999999999999996E-3</v>
       </c>
       <c r="E30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.68246213387612298</v>
+        <v>6.8999999999999999E-3</v>
       </c>
       <c r="F30">
-        <f t="shared" ca="1" si="9"/>
-        <v>8.4300259559227597E-2</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="G30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.8510177614821306</v>
+        <v>7.1000000000000004E-3</v>
       </c>
       <c r="H30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.70786205880811481</v>
+        <v>7.1999999999999998E-3</v>
       </c>
       <c r="I30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.10045427695553721</v>
+        <v>7.3000000000000001E-3</v>
       </c>
       <c r="J30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.3484268077353353</v>
+        <v>7.4000000000000003E-3</v>
       </c>
       <c r="K30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.79747706995973167</v>
+        <v>7.4999999999999997E-3</v>
       </c>
       <c r="L30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.56341775754542944</v>
+        <v>7.5500000000000003E-3</v>
       </c>
       <c r="M30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.97542467492953178</v>
+        <v>7.6E-3</v>
       </c>
       <c r="N30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.3819625859787652</v>
+        <v>7.6499999999999997E-3</v>
       </c>
       <c r="O30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.11808170606109303</v>
+        <v>7.7000000000000002E-3</v>
       </c>
       <c r="P30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.50859808957797037</v>
+        <v>7.7499999999999999E-3</v>
       </c>
       <c r="Q30">
-        <f t="shared" ca="1" si="9"/>
-        <v>0.21988592180736355</v>
+        <v>7.7999999999999996E-3</v>
       </c>
       <c r="R30">
-        <f t="shared" ca="1" si="10"/>
-        <v>0.61352841899286936</v>
+        <v>7.8499999999999993E-3</v>
       </c>
       <c r="S30">
-        <f t="shared" ca="1" si="10"/>
-        <v>0.86814654592186657</v>
+        <v>7.9000000000000008E-3</v>
       </c>
       <c r="T30">
-        <f t="shared" ca="1" si="10"/>
-        <v>0.10755148378222612</v>
+        <v>7.9500000000000005E-3</v>
       </c>
       <c r="U30">
-        <f t="shared" ca="1" si="10"/>
-        <v>0.69886661853005705</v>
+        <v>8.0000000000000002E-3</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.3">
@@ -5715,347 +5448,267 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B33">
-        <f t="shared" ref="B33:Q36" ca="1" si="11">RAND()</f>
-        <v>0.2634511635444966</v>
+        <v>2.1399999999999999E-2</v>
       </c>
       <c r="C33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.4463431608790589</v>
+        <v>2.1600000000000001E-2</v>
       </c>
       <c r="D33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.70657141913060417</v>
+        <v>2.1700000000000001E-2</v>
       </c>
       <c r="E33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.24433142676032149</v>
+        <v>2.18E-2</v>
       </c>
       <c r="F33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.43080012376299925</v>
+        <v>2.1899999999999999E-2</v>
       </c>
       <c r="G33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.71352361632608918</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="H33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.34005440264391651</v>
+        <v>2.2100000000000002E-2</v>
       </c>
       <c r="I33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.64216999517685902</v>
+        <v>2.2200000000000001E-2</v>
       </c>
       <c r="J33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.8702032287094642</v>
+        <v>2.23E-2</v>
       </c>
       <c r="K33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.33246818839868042</v>
+        <v>2.24E-2</v>
       </c>
       <c r="L33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.64536701163164323</v>
+        <v>2.2450000000000001E-2</v>
       </c>
       <c r="M33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.65058925503219722</v>
+        <v>2.2499999999999999E-2</v>
       </c>
       <c r="N33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.39520471785370215</v>
+        <v>2.2550000000000001E-2</v>
       </c>
       <c r="O33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.88238127239727049</v>
+        <v>2.2599999999999999E-2</v>
       </c>
       <c r="P33">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.13463568534008441</v>
+        <v>2.265E-2</v>
       </c>
       <c r="Q33">
-        <f t="shared" ca="1" si="11"/>
-        <v>3.0403962907946225E-2</v>
+        <v>2.2700000000000001E-2</v>
       </c>
       <c r="R33">
-        <f t="shared" ref="R33:U36" ca="1" si="12">RAND()</f>
-        <v>0.65220534625959348</v>
+        <v>2.2749999999999999E-2</v>
       </c>
       <c r="S33">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.98335713268441283</v>
+        <v>2.2800000000000001E-2</v>
       </c>
       <c r="T33">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.26541324930745136</v>
+        <v>2.2849999999999999E-2</v>
       </c>
       <c r="U33">
-        <f t="shared" ca="1" si="12"/>
-        <v>6.4855035469933098E-2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
+        <v>2.29E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.65861206988009846</v>
+        <v>1.9599999999999999E-2</v>
       </c>
       <c r="C34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.6120927366333232</v>
+        <v>1.9800000000000002E-2</v>
       </c>
       <c r="D34">
-        <f t="shared" ca="1" si="11"/>
-        <v>4.3503797082272921E-2</v>
+        <v>1.9900000000000001E-2</v>
       </c>
       <c r="E34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.45424005200862849</v>
+        <v>0.02</v>
       </c>
       <c r="F34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.51512152829123181</v>
+        <v>2.01E-2</v>
       </c>
       <c r="G34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.25998102799536293</v>
+        <v>2.0199999999999999E-2</v>
       </c>
       <c r="H34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.2814042808224605</v>
+        <v>2.0299999999999999E-2</v>
       </c>
       <c r="I34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.31204611425582152</v>
+        <v>2.0400000000000001E-2</v>
       </c>
       <c r="J34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.52475395022722771</v>
+        <v>2.0500000000000001E-2</v>
       </c>
       <c r="K34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.64312989459403247</v>
+        <v>2.06E-2</v>
       </c>
       <c r="L34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.69134569109698074</v>
+        <v>2.0650000000000002E-2</v>
       </c>
       <c r="M34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.71510220992878526</v>
+        <v>2.07E-2</v>
       </c>
       <c r="N34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.5039163844293979</v>
+        <v>2.0750000000000001E-2</v>
       </c>
       <c r="O34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.83447538751899919</v>
+        <v>2.0799999999999999E-2</v>
       </c>
       <c r="P34">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.81279637634634183</v>
+        <v>2.085E-2</v>
       </c>
       <c r="Q34">
-        <f t="shared" ca="1" si="11"/>
-        <v>3.7267947777835153E-2</v>
+        <v>2.0899999999999998E-2</v>
       </c>
       <c r="R34">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.23215656683986641</v>
+        <v>2.095E-2</v>
       </c>
       <c r="S34">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.21136315709749154</v>
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="T34">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.41054547023373722</v>
+        <v>2.1049999999999999E-2</v>
       </c>
       <c r="U34">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.32131552829721832</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
+        <v>2.1100000000000001E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.16952758299547455</v>
-      </c>
-      <c r="C35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.89388600643893024</v>
-      </c>
-      <c r="D35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.91217695500656182</v>
-      </c>
-      <c r="E35">
-        <f t="shared" ca="1" si="11"/>
-        <v>7.5736230114858305E-2</v>
-      </c>
-      <c r="F35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.33775992264538013</v>
-      </c>
-      <c r="G35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.84231309579038649</v>
-      </c>
-      <c r="H35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.18433247814230891</v>
-      </c>
-      <c r="I35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.51793959810063128</v>
-      </c>
-      <c r="J35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.84455510333793782</v>
-      </c>
-      <c r="K35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.3492378383107948</v>
-      </c>
-      <c r="L35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.42609446193086431</v>
-      </c>
-      <c r="M35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.12823615588780668</v>
-      </c>
-      <c r="N35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.51682758308182353</v>
-      </c>
-      <c r="O35">
-        <f t="shared" ca="1" si="11"/>
-        <v>3.0802476165482373E-3</v>
-      </c>
-      <c r="P35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.72217937124338205</v>
-      </c>
-      <c r="Q35">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.16458460566310207</v>
-      </c>
-      <c r="R35">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.47699913200226185</v>
-      </c>
-      <c r="S35">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.75615239683645741</v>
-      </c>
-      <c r="T35">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.83390251894015988</v>
-      </c>
-      <c r="U35">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.76859695945976114</v>
-      </c>
-    </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B35" s="8">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="C35" s="8">
+        <v>2.12E-2</v>
+      </c>
+      <c r="D35" s="8">
+        <v>2.1299999999999999E-2</v>
+      </c>
+      <c r="E35" s="8">
+        <v>2.1399999999999999E-2</v>
+      </c>
+      <c r="F35" s="8">
+        <v>2.1499999999999998E-2</v>
+      </c>
+      <c r="G35" s="8">
+        <v>2.1600000000000001E-2</v>
+      </c>
+      <c r="H35" s="8">
+        <v>2.1700000000000001E-2</v>
+      </c>
+      <c r="I35" s="8">
+        <v>2.18E-2</v>
+      </c>
+      <c r="J35" s="8">
+        <v>2.1899999999999999E-2</v>
+      </c>
+      <c r="K35" s="8">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="L35" s="8">
+        <v>2.205E-2</v>
+      </c>
+      <c r="M35" s="8">
+        <v>2.2100000000000002E-2</v>
+      </c>
+      <c r="N35" s="8">
+        <v>2.215E-2</v>
+      </c>
+      <c r="O35" s="8">
+        <v>2.2200000000000001E-2</v>
+      </c>
+      <c r="P35" s="8">
+        <v>2.2249999999999999E-2</v>
+      </c>
+      <c r="Q35" s="8">
+        <v>2.23E-2</v>
+      </c>
+      <c r="R35" s="8">
+        <v>2.2349999999999998E-2</v>
+      </c>
+      <c r="S35" s="8">
+        <v>2.24E-2</v>
+      </c>
+      <c r="T35" s="8">
+        <v>2.2450000000000001E-2</v>
+      </c>
+      <c r="U35" s="8">
+        <v>2.2499999999999999E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.94985306809239678</v>
-      </c>
-      <c r="C36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.30972377122713579</v>
-      </c>
-      <c r="D36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.54183490229249254</v>
-      </c>
-      <c r="E36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.71472035209710028</v>
-      </c>
-      <c r="F36">
-        <f t="shared" ca="1" si="11"/>
-        <v>9.5305584647929709E-2</v>
-      </c>
-      <c r="G36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.82667617956994532</v>
-      </c>
-      <c r="H36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.74796105154779358</v>
-      </c>
-      <c r="I36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.57852649591102978</v>
-      </c>
-      <c r="J36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.74218905026510495</v>
-      </c>
-      <c r="K36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.12021201655803782</v>
-      </c>
-      <c r="L36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.86082952374411537</v>
-      </c>
-      <c r="M36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.87524418251320235</v>
-      </c>
-      <c r="N36">
-        <f t="shared" ca="1" si="11"/>
-        <v>6.9070581112578466E-2</v>
-      </c>
-      <c r="O36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.60717577720977822</v>
-      </c>
-      <c r="P36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.69012769632312176</v>
-      </c>
-      <c r="Q36">
-        <f t="shared" ca="1" si="11"/>
-        <v>0.29262923959210463</v>
-      </c>
-      <c r="R36">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.93956076709133196</v>
-      </c>
-      <c r="S36">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.10927441410059446</v>
-      </c>
-      <c r="T36">
-        <f t="shared" ca="1" si="12"/>
-        <v>0.67806700068193104</v>
-      </c>
-      <c r="U36">
-        <f t="shared" ca="1" si="12"/>
-        <v>4.8665905693893174E-3</v>
-      </c>
-    </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B36" s="8">
+        <v>6.4999999999999997E-3</v>
+      </c>
+      <c r="C36" s="8">
+        <v>6.7000000000000002E-3</v>
+      </c>
+      <c r="D36" s="8">
+        <v>6.7999999999999996E-3</v>
+      </c>
+      <c r="E36" s="8">
+        <v>6.8999999999999999E-3</v>
+      </c>
+      <c r="F36" s="8">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="G36" s="8">
+        <v>7.1000000000000004E-3</v>
+      </c>
+      <c r="H36" s="8">
+        <v>7.1999999999999998E-3</v>
+      </c>
+      <c r="I36" s="8">
+        <v>7.3000000000000001E-3</v>
+      </c>
+      <c r="J36" s="8">
+        <v>7.4000000000000003E-3</v>
+      </c>
+      <c r="K36" s="8">
+        <v>7.4999999999999997E-3</v>
+      </c>
+      <c r="L36" s="8">
+        <v>7.5500000000000003E-3</v>
+      </c>
+      <c r="M36" s="8">
+        <v>7.6E-3</v>
+      </c>
+      <c r="N36" s="8">
+        <v>7.6499999999999997E-3</v>
+      </c>
+      <c r="O36" s="8">
+        <v>7.7000000000000002E-3</v>
+      </c>
+      <c r="P36" s="8">
+        <v>7.7499999999999999E-3</v>
+      </c>
+      <c r="Q36" s="8">
+        <v>7.7999999999999996E-3</v>
+      </c>
+      <c r="R36" s="8">
+        <v>7.8499999999999993E-3</v>
+      </c>
+      <c r="S36" s="8">
+        <v>7.9000000000000008E-3</v>
+      </c>
+      <c r="T36" s="8">
+        <v>7.9500000000000005E-3</v>
+      </c>
+      <c r="U36" s="8">
+        <v>8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>39</v>
       </c>
@@ -6120,1285 +5773,1122 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B38">
-        <f t="shared" ref="B38:Q44" ca="1" si="13">RAND()</f>
-        <v>0.26679942536692691</v>
+        <v>-1.34E-2</v>
       </c>
       <c r="C38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.31112087465104943</v>
+        <v>-1.32E-2</v>
       </c>
       <c r="D38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.24565014697156895</v>
+        <v>-1.3100000000000001E-2</v>
       </c>
       <c r="E38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.37673716819142467</v>
+        <v>-1.2999999999999999E-2</v>
       </c>
       <c r="F38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.13724742986023186</v>
+        <v>-1.29E-2</v>
       </c>
       <c r="G38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.95793518970822689</v>
+        <v>-1.2800000000000001E-2</v>
       </c>
       <c r="H38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.68971196738140084</v>
+        <v>-1.2699999999999999E-2</v>
       </c>
       <c r="I38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.98855278074487063</v>
+        <v>-1.26E-2</v>
       </c>
       <c r="J38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.41025688672679395</v>
+        <v>-1.2500000000000001E-2</v>
       </c>
       <c r="K38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.55551219563208365</v>
+        <v>-1.24E-2</v>
       </c>
       <c r="L38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.84718484578251829</v>
+        <v>-1.235E-2</v>
       </c>
       <c r="M38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.74982472821819468</v>
+        <v>-1.23E-2</v>
       </c>
       <c r="N38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.75430661742919258</v>
+        <v>-1.225E-2</v>
       </c>
       <c r="O38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.805150246156215</v>
+        <v>-1.2200000000000001E-2</v>
       </c>
       <c r="P38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.83333387605190279</v>
+        <v>-1.2149999999999999E-2</v>
       </c>
       <c r="Q38">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.30800057010565052</v>
+        <v>-1.21E-2</v>
       </c>
       <c r="R38">
-        <f t="shared" ref="R38:U44" ca="1" si="14">RAND()</f>
-        <v>0.1536674584031229</v>
+        <v>-1.205E-2</v>
       </c>
       <c r="S38">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.47282963702374059</v>
+        <v>-1.2E-2</v>
       </c>
       <c r="T38">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.15792337415848989</v>
+        <v>-1.1950000000000001E-2</v>
       </c>
       <c r="U38">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.1609506786443341</v>
-      </c>
-    </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
+        <v>-1.1900000000000001E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.2523695863127362</v>
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="C39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.10318002838788276</v>
+        <v>2.12E-2</v>
       </c>
       <c r="D39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.98761262522388105</v>
+        <v>2.1299999999999999E-2</v>
       </c>
       <c r="E39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.44860819495377657</v>
+        <v>2.1399999999999999E-2</v>
       </c>
       <c r="F39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.57635163155754454</v>
+        <v>2.1499999999999998E-2</v>
       </c>
       <c r="G39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.50119382505249466</v>
+        <v>2.1600000000000001E-2</v>
       </c>
       <c r="H39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.50296575408880662</v>
+        <v>2.1700000000000001E-2</v>
       </c>
       <c r="I39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.85405327557605193</v>
+        <v>2.18E-2</v>
       </c>
       <c r="J39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.94761715342655095</v>
+        <v>2.1899999999999999E-2</v>
       </c>
       <c r="K39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.66168543049887185</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="L39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.34048933196064735</v>
+        <v>2.205E-2</v>
       </c>
       <c r="M39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.96155336346944564</v>
+        <v>2.2100000000000002E-2</v>
       </c>
       <c r="N39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.7758690545527982</v>
+        <v>2.215E-2</v>
       </c>
       <c r="O39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.67694076377886103</v>
+        <v>2.2200000000000001E-2</v>
       </c>
       <c r="P39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.59099689876827166</v>
+        <v>2.2249999999999999E-2</v>
       </c>
       <c r="Q39">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.39799188307921696</v>
+        <v>2.23E-2</v>
       </c>
       <c r="R39">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.90176682810591546</v>
+        <v>2.2349999999999998E-2</v>
       </c>
       <c r="S39">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.37648774869764345</v>
+        <v>2.24E-2</v>
       </c>
       <c r="T39">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.62707383727811505</v>
+        <v>2.2450000000000001E-2</v>
       </c>
       <c r="U39">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.28978446611100284</v>
-      </c>
-    </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
+        <v>2.2499999999999999E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>43</v>
       </c>
       <c r="B40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.49679124154815968</v>
+        <v>0.01</v>
       </c>
       <c r="C40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.58667709567303239</v>
+        <v>1.0500000000000001E-2</v>
       </c>
       <c r="D40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.99220057092384784</v>
+        <v>1.066666666666667E-2</v>
       </c>
       <c r="E40">
-        <f t="shared" ca="1" si="13"/>
-        <v>3.3171239476036729E-2</v>
+        <v>1.083333333333333E-2</v>
       </c>
       <c r="F40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.71525172920618507</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="G40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.87971762590169489</v>
+        <v>1.12E-2</v>
       </c>
       <c r="H40">
-        <f t="shared" ca="1" si="13"/>
-        <v>5.8082446275473765E-2</v>
+        <v>1.14E-2</v>
       </c>
       <c r="I40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.50842901241909932</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="J40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.68822435606082633</v>
+        <v>1.18E-2</v>
       </c>
       <c r="K40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.80312478478885185</v>
+        <v>1.2E-2</v>
       </c>
       <c r="L40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.27751397283304069</v>
+        <v>1.21E-2</v>
       </c>
       <c r="M40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.13328360600066702</v>
+        <v>1.2200000000000001E-2</v>
       </c>
       <c r="N40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.45155419473246716</v>
+        <v>1.23E-2</v>
       </c>
       <c r="O40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.46206036157560471</v>
+        <v>1.24E-2</v>
       </c>
       <c r="P40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.42931822704603662</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="Q40">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.93936551827421977</v>
+        <v>1.26E-2</v>
       </c>
       <c r="R40">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.66583615578444444</v>
+        <v>1.2699999999999999E-2</v>
       </c>
       <c r="S40">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.89893940511295212</v>
+        <v>1.2800000000000001E-2</v>
       </c>
       <c r="T40">
-        <f t="shared" ca="1" si="14"/>
-        <v>5.8670796596195784E-2</v>
+        <v>1.29E-2</v>
       </c>
       <c r="U40">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.39153241797302818</v>
-      </c>
-    </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
+        <v>1.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>44</v>
       </c>
       <c r="B41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.34929796014151215</v>
+        <v>1.2E-2</v>
       </c>
       <c r="C41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.39498481137015351</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="D41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.76940494212142518</v>
+        <v>1.266666666666667E-2</v>
       </c>
       <c r="E41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.33486355111356347</v>
+        <v>1.2833333333333329E-2</v>
       </c>
       <c r="F41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.55350794820010152</v>
+        <v>1.2999999999999999E-2</v>
       </c>
       <c r="G41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.25371269339706204</v>
+        <v>1.32E-2</v>
       </c>
       <c r="H41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.80358997611133498</v>
+        <v>1.34E-2</v>
       </c>
       <c r="I41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.85752475893320246</v>
+        <v>1.3599999999999999E-2</v>
       </c>
       <c r="J41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.20791712351005032</v>
+        <v>1.38E-2</v>
       </c>
       <c r="K41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.82530745708260622</v>
+        <v>1.4E-2</v>
       </c>
       <c r="L41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.95118981945401282</v>
+        <v>1.41E-2</v>
       </c>
       <c r="M41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.50046047813422845</v>
+        <v>1.4200000000000001E-2</v>
       </c>
       <c r="N41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.58006083919708284</v>
+        <v>1.43E-2</v>
       </c>
       <c r="O41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.8268935795539748</v>
+        <v>1.44E-2</v>
       </c>
       <c r="P41">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.91560236186893895</v>
+        <v>1.4500000000000001E-2</v>
       </c>
       <c r="Q41">
-        <f t="shared" ca="1" si="13"/>
-        <v>3.6383542810021097E-2</v>
+        <v>1.46E-2</v>
       </c>
       <c r="R41">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.9274753200136624</v>
+        <v>1.47E-2</v>
       </c>
       <c r="S41">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.89601077555076858</v>
+        <v>1.4800000000000001E-2</v>
       </c>
       <c r="T41">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.83856103125758297</v>
+        <v>1.49E-2</v>
       </c>
       <c r="U41">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.40408102203359908</v>
-      </c>
-    </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.3">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="W41" s="7"/>
+      <c r="X41" s="7"/>
+      <c r="Y41" s="7"/>
+      <c r="Z41" s="7"/>
+      <c r="AA41" s="7"/>
+      <c r="AB41" s="7"/>
+    </row>
+    <row r="42" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>45</v>
       </c>
       <c r="B42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.622934815091161</v>
+        <v>1.4E-2</v>
       </c>
       <c r="C42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.9572771644618191</v>
+        <v>1.4500000000000001E-2</v>
       </c>
       <c r="D42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.2513602446569112</v>
+        <v>1.4666666666666672E-2</v>
       </c>
       <c r="E42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.32427962130893151</v>
+        <v>1.4833333333333329E-2</v>
       </c>
       <c r="F42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.96844895224285976</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="G42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.28295965450109528</v>
+        <v>1.52E-2</v>
       </c>
       <c r="H42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.43378693975686444</v>
+        <v>1.54E-2</v>
       </c>
       <c r="I42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.16542129287589458</v>
+        <v>1.5599999999999999E-2</v>
       </c>
       <c r="J42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.48202666825036267</v>
+        <v>1.5800000000000002E-2</v>
       </c>
       <c r="K42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.85860869072119295</v>
+        <v>1.6E-2</v>
       </c>
       <c r="L42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.22299410061278702</v>
+        <v>1.61E-2</v>
       </c>
       <c r="M42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.79459977711518115</v>
+        <v>1.6199999999999999E-2</v>
       </c>
       <c r="N42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.55719967577960539</v>
+        <v>1.6299999999999999E-2</v>
       </c>
       <c r="O42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.88576766870446211</v>
+        <v>1.6400000000000001E-2</v>
       </c>
       <c r="P42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.62487594830182214</v>
+        <v>1.6500000000000001E-2</v>
       </c>
       <c r="Q42">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.23605814634334976</v>
+        <v>1.66E-2</v>
       </c>
       <c r="R42">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.63427492263368779</v>
+        <v>1.67E-2</v>
       </c>
       <c r="S42">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.62474285140185326</v>
+        <v>1.6799999999999999E-2</v>
       </c>
       <c r="T42">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.82179065477848356</v>
+        <v>1.6899999999999998E-2</v>
       </c>
       <c r="U42">
-        <f t="shared" ca="1" si="14"/>
-        <v>3.2944468612008726E-2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
+        <v>1.7000000000000001E-2</v>
+      </c>
+      <c r="W42" s="7"/>
+      <c r="X42" s="7"/>
+      <c r="Y42" s="7"/>
+      <c r="Z42" s="7"/>
+      <c r="AA42" s="7"/>
+      <c r="AB42" s="7"/>
+    </row>
+    <row r="43" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
         <v>46</v>
       </c>
       <c r="B43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.9079524015753021</v>
+        <v>1.6E-2</v>
       </c>
       <c r="C43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.351778264982616</v>
+        <v>1.6500000000000001E-2</v>
       </c>
       <c r="D43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.69212222588374295</v>
+        <v>1.666666666666667E-2</v>
       </c>
       <c r="E43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.21494620275516607</v>
+        <v>1.6833333333333329E-2</v>
       </c>
       <c r="F43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.11112276493928874</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="G43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.11541833033325322</v>
+        <v>1.72E-2</v>
       </c>
       <c r="H43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.24132793348960979</v>
+        <v>1.7399999999999999E-2</v>
       </c>
       <c r="I43">
-        <f t="shared" ca="1" si="13"/>
-        <v>5.5463836993736582E-2</v>
+        <v>1.7600000000000001E-2</v>
       </c>
       <c r="J43">
-        <f t="shared" ca="1" si="13"/>
-        <v>3.9270799944444712E-2</v>
+        <v>1.78E-2</v>
       </c>
       <c r="K43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.36525435747758861</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="L43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.98698216178536768</v>
+        <v>1.8100000000000002E-2</v>
       </c>
       <c r="M43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.61233187269241185</v>
+        <v>1.8200000000000001E-2</v>
       </c>
       <c r="N43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.45938235374447633</v>
+        <v>1.83E-2</v>
       </c>
       <c r="O43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.97955716221504863</v>
+        <v>1.84E-2</v>
       </c>
       <c r="P43">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.86222181299559963</v>
+        <v>1.8499999999999999E-2</v>
       </c>
       <c r="Q43">
-        <f t="shared" ca="1" si="13"/>
-        <v>8.5046450192737932E-2</v>
+        <v>1.8599999999999998E-2</v>
       </c>
       <c r="R43">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.38447322941256012</v>
+        <v>1.8700000000000001E-2</v>
       </c>
       <c r="S43">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.52386791548415734</v>
+        <v>1.8800000000000001E-2</v>
       </c>
       <c r="T43">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.1608754839813693</v>
+        <v>1.89E-2</v>
       </c>
       <c r="U43">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.51168085630377913</v>
-      </c>
-    </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
+        <v>1.9E-2</v>
+      </c>
+      <c r="W43" s="7"/>
+      <c r="X43" s="7"/>
+      <c r="Y43" s="7"/>
+      <c r="Z43" s="7"/>
+      <c r="AA43" s="7"/>
+      <c r="AB43" s="7"/>
+    </row>
+    <row r="44" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>47</v>
       </c>
       <c r="B44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.79808094825767184</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="C44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.16325158981660515</v>
+        <v>1.8499999999999999E-2</v>
       </c>
       <c r="D44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.27633808934508974</v>
+        <v>1.8666666666666672E-2</v>
       </c>
       <c r="E44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.57885540060009655</v>
+        <v>1.8833333333333327E-2</v>
       </c>
       <c r="F44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.23328206783492444</v>
+        <v>1.9E-2</v>
       </c>
       <c r="G44">
-        <f t="shared" ca="1" si="13"/>
-        <v>1.7270907195652385E-2</v>
+        <v>1.9199999999999998E-2</v>
       </c>
       <c r="H44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.25406225119623571</v>
+        <v>1.9400000000000001E-2</v>
       </c>
       <c r="I44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.98484967897832199</v>
+        <v>1.9599999999999999E-2</v>
       </c>
       <c r="J44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.46716593029023323</v>
+        <v>1.9800000000000002E-2</v>
       </c>
       <c r="K44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.42428853904915487</v>
+        <v>0.02</v>
       </c>
       <c r="L44">
-        <f t="shared" ca="1" si="13"/>
-        <v>3.641620786339006E-3</v>
+        <v>2.01E-2</v>
       </c>
       <c r="M44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.18947220096105999</v>
+        <v>2.0199999999999999E-2</v>
       </c>
       <c r="N44">
-        <f t="shared" ca="1" si="13"/>
-        <v>2.375329903846557E-2</v>
+        <v>2.0299999999999999E-2</v>
       </c>
       <c r="O44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.47859556926507718</v>
+        <v>2.0400000000000001E-2</v>
       </c>
       <c r="P44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.40158272045132348</v>
+        <v>2.0500000000000001E-2</v>
       </c>
       <c r="Q44">
-        <f t="shared" ca="1" si="13"/>
-        <v>0.76500266925456362</v>
+        <v>2.06E-2</v>
       </c>
       <c r="R44">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.51557972022697385</v>
+        <v>2.07E-2</v>
       </c>
       <c r="S44">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.12345726161432991</v>
+        <v>2.0799999999999999E-2</v>
       </c>
       <c r="T44">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.16458215901005457</v>
+        <v>2.0899999999999998E-2</v>
       </c>
       <c r="U44">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.96497478368177803</v>
-      </c>
-    </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="W44" s="7"/>
+      <c r="X44" s="7"/>
+      <c r="Y44" s="7"/>
+      <c r="Z44" s="7"/>
+      <c r="AA44" s="7"/>
+      <c r="AB44" s="7"/>
+    </row>
+    <row r="45" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>48</v>
       </c>
       <c r="B45" s="4">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="C45" s="4">
-        <v>0</v>
+        <v>2.0500000000000001E-2</v>
       </c>
       <c r="D45" s="4">
-        <v>0</v>
+        <v>2.066666666666667E-2</v>
       </c>
       <c r="E45" s="4">
-        <v>0</v>
+        <v>2.0833333333333329E-2</v>
       </c>
       <c r="F45" s="4">
-        <v>0</v>
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="G45" s="4">
-        <v>0</v>
+        <v>2.12E-2</v>
       </c>
       <c r="H45" s="4">
-        <v>0</v>
+        <v>2.1399999999999999E-2</v>
       </c>
       <c r="I45" s="4">
-        <v>0</v>
+        <v>2.1600000000000001E-2</v>
       </c>
       <c r="J45" s="4">
-        <v>0</v>
+        <v>2.18E-2</v>
       </c>
       <c r="K45" s="4">
-        <v>0</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="L45" s="4">
-        <v>0</v>
+        <v>2.2100000000000002E-2</v>
       </c>
       <c r="M45" s="4">
-        <v>0</v>
+        <v>2.2200000000000001E-2</v>
       </c>
       <c r="N45" s="4">
-        <v>0</v>
+        <v>2.23E-2</v>
       </c>
       <c r="O45" s="4">
-        <v>0</v>
+        <v>2.24E-2</v>
       </c>
       <c r="P45" s="4">
-        <v>0</v>
+        <v>2.2499999999999999E-2</v>
       </c>
       <c r="Q45" s="4">
-        <v>0</v>
+        <v>2.2599999999999999E-2</v>
       </c>
       <c r="R45" s="4">
-        <v>0</v>
+        <v>2.2700000000000001E-2</v>
       </c>
       <c r="S45" s="4">
-        <v>0</v>
+        <v>2.2800000000000001E-2</v>
       </c>
       <c r="T45" s="4">
-        <v>0</v>
+        <v>2.29E-2</v>
       </c>
       <c r="U45" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
+        <v>2.3E-2</v>
+      </c>
+      <c r="W45" s="7"/>
+      <c r="X45" s="7"/>
+      <c r="Y45" s="7"/>
+      <c r="Z45" s="7"/>
+      <c r="AA45" s="7"/>
+      <c r="AB45" s="7"/>
+    </row>
+    <row r="46" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>49</v>
       </c>
       <c r="B46" s="4">
-        <v>0</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="C46" s="4">
-        <v>0</v>
+        <v>2.2499999999999999E-2</v>
       </c>
       <c r="D46" s="4">
-        <v>0</v>
+        <v>2.2666666666666672E-2</v>
       </c>
       <c r="E46" s="4">
-        <v>0</v>
+        <v>2.2833333333333327E-2</v>
       </c>
       <c r="F46" s="4">
-        <v>0</v>
+        <v>2.3E-2</v>
       </c>
       <c r="G46" s="4">
-        <v>0</v>
+        <v>2.3199999999999998E-2</v>
       </c>
       <c r="H46" s="4">
-        <v>0</v>
+        <v>2.3400000000000001E-2</v>
       </c>
       <c r="I46" s="4">
-        <v>0</v>
+        <v>2.3599999999999999E-2</v>
       </c>
       <c r="J46" s="4">
-        <v>0</v>
+        <v>2.3800000000000002E-2</v>
       </c>
       <c r="K46" s="4">
-        <v>0</v>
+        <v>2.4E-2</v>
       </c>
       <c r="L46" s="4">
-        <v>0</v>
+        <v>2.41E-2</v>
       </c>
       <c r="M46" s="4">
-        <v>0</v>
+        <v>2.4199999999999999E-2</v>
       </c>
       <c r="N46" s="4">
-        <v>0</v>
+        <v>2.4299999999999999E-2</v>
       </c>
       <c r="O46" s="4">
-        <v>0</v>
+        <v>2.4400000000000002E-2</v>
       </c>
       <c r="P46" s="4">
-        <v>0</v>
+        <v>2.4500000000000001E-2</v>
       </c>
       <c r="Q46" s="4">
-        <v>0</v>
+        <v>2.46E-2</v>
       </c>
       <c r="R46" s="4">
-        <v>0</v>
+        <v>2.47E-2</v>
       </c>
       <c r="S46" s="4">
-        <v>0</v>
+        <v>2.4799999999999999E-2</v>
       </c>
       <c r="T46" s="4">
-        <v>0</v>
+        <v>2.4899999999999999E-2</v>
       </c>
       <c r="U46" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="W46" s="7"/>
+      <c r="X46" s="7"/>
+      <c r="Y46" s="7"/>
+      <c r="Z46" s="7"/>
+      <c r="AA46" s="7"/>
+      <c r="AB46" s="7"/>
+    </row>
+    <row r="47" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>50</v>
       </c>
       <c r="B47">
-        <f t="shared" ref="B47:Q51" ca="1" si="15">RAND()</f>
-        <v>6.7765916272566229E-2</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="C47">
-        <f t="shared" ca="1" si="15"/>
-        <v>7.8683206913990777E-2</v>
+        <v>8.5000000000000006E-3</v>
       </c>
       <c r="D47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.33204122904657363</v>
+        <v>8.666666666666668E-3</v>
       </c>
       <c r="E47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.91665269087378476</v>
+        <v>8.8333333333333337E-3</v>
       </c>
       <c r="F47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.74771176012747331</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="G47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.6826329705711357</v>
+        <v>9.1999999999999998E-3</v>
       </c>
       <c r="H47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.16510529360690174</v>
+        <v>9.4000000000000004E-3</v>
       </c>
       <c r="I47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.63644151860991904</v>
+        <v>9.5999999999999992E-3</v>
       </c>
       <c r="J47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.65291219332593542</v>
+        <v>9.7999999999999997E-3</v>
       </c>
       <c r="K47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.89092495178483966</v>
+        <v>0.01</v>
       </c>
       <c r="L47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.38890032124280272</v>
+        <v>1.01E-2</v>
       </c>
       <c r="M47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.46001174677204826</v>
+        <v>1.0200000000000001E-2</v>
       </c>
       <c r="N47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.10907162223484801</v>
+        <v>1.03E-2</v>
       </c>
       <c r="O47">
-        <f t="shared" ca="1" si="15"/>
-        <v>4.9897612687668347E-2</v>
+        <v>1.04E-2</v>
       </c>
       <c r="P47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.63053972504960631</v>
+        <v>1.0500000000000001E-2</v>
       </c>
       <c r="Q47">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.77253662409136514</v>
+        <v>1.06E-2</v>
       </c>
       <c r="R47">
-        <f t="shared" ref="R47:U51" ca="1" si="16">RAND()</f>
-        <v>0.95836631421064999</v>
+        <v>1.0699999999999999E-2</v>
       </c>
       <c r="S47">
-        <f t="shared" ca="1" si="16"/>
-        <v>4.1131826313015596E-2</v>
+        <v>1.0800000000000001E-2</v>
       </c>
       <c r="T47">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.62341330476019208</v>
+        <v>1.09E-2</v>
       </c>
       <c r="U47">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.48242183146205952</v>
-      </c>
-    </row>
-    <row r="48" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="W47" s="7"/>
+    </row>
+    <row r="48" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
         <v>51</v>
       </c>
       <c r="B48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.44201850196230619</v>
+        <v>0.01</v>
       </c>
       <c r="C48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.11222622979281061</v>
+        <v>1.0500000000000001E-2</v>
       </c>
       <c r="D48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.22824943759719218</v>
+        <v>1.066666666666667E-2</v>
       </c>
       <c r="E48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.91782106009600628</v>
+        <v>1.083333333333333E-2</v>
       </c>
       <c r="F48">
-        <f t="shared" ca="1" si="15"/>
-        <v>8.9774856826118188E-2</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="G48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.3463097178806156</v>
+        <v>1.12E-2</v>
       </c>
       <c r="H48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.51182677824376144</v>
+        <v>1.14E-2</v>
       </c>
       <c r="I48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.65387281057705149</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="J48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.49454030593053189</v>
+        <v>1.18E-2</v>
       </c>
       <c r="K48">
-        <f t="shared" ca="1" si="15"/>
-        <v>7.8298834645999627E-2</v>
+        <v>1.2E-2</v>
       </c>
       <c r="L48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.26053488051109241</v>
+        <v>1.21E-2</v>
       </c>
       <c r="M48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.12759184685681768</v>
+        <v>1.2200000000000001E-2</v>
       </c>
       <c r="N48">
-        <f t="shared" ca="1" si="15"/>
-        <v>4.0671159807036728E-2</v>
+        <v>1.23E-2</v>
       </c>
       <c r="O48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.67455362569455157</v>
+        <v>1.24E-2</v>
       </c>
       <c r="P48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.20663090735082157</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="Q48">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.92147928735602425</v>
+        <v>1.26E-2</v>
       </c>
       <c r="R48">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.14126790376043297</v>
+        <v>1.2699999999999999E-2</v>
       </c>
       <c r="S48">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.78267731500557969</v>
+        <v>1.2800000000000001E-2</v>
       </c>
       <c r="T48">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.27769706369675917</v>
+        <v>1.29E-2</v>
       </c>
       <c r="U48">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.73248637531159122</v>
-      </c>
-    </row>
-    <row r="49" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="W48" s="7"/>
+      <c r="X48" s="7"/>
+      <c r="Y48" s="7"/>
+      <c r="Z48" s="7"/>
+      <c r="AA48" s="7"/>
+      <c r="AB48" s="7"/>
+    </row>
+    <row r="49" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
         <v>52</v>
       </c>
       <c r="B49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.14304878505491991</v>
+        <v>1.2E-2</v>
       </c>
       <c r="C49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.26302265889258902</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="D49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.29807811558755826</v>
+        <v>1.266666666666667E-2</v>
       </c>
       <c r="E49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.35335050532531298</v>
+        <v>1.2833333333333329E-2</v>
       </c>
       <c r="F49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.19827369203000011</v>
+        <v>1.2999999999999999E-2</v>
       </c>
       <c r="G49">
-        <f t="shared" ca="1" si="15"/>
-        <v>4.6588525681797388E-2</v>
+        <v>1.32E-2</v>
       </c>
       <c r="H49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.57464789544360995</v>
+        <v>1.34E-2</v>
       </c>
       <c r="I49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.45192639460546546</v>
+        <v>1.3599999999999999E-2</v>
       </c>
       <c r="J49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.5404591940546144</v>
+        <v>1.38E-2</v>
       </c>
       <c r="K49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.68790744237848589</v>
+        <v>1.4E-2</v>
       </c>
       <c r="L49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.13038410907771525</v>
+        <v>1.41E-2</v>
       </c>
       <c r="M49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.98493872885520539</v>
+        <v>1.4200000000000001E-2</v>
       </c>
       <c r="N49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.26403551750874688</v>
+        <v>1.43E-2</v>
       </c>
       <c r="O49">
-        <f t="shared" ca="1" si="15"/>
-        <v>9.3510702261641931E-2</v>
+        <v>1.44E-2</v>
       </c>
       <c r="P49">
-        <f t="shared" ca="1" si="15"/>
-        <v>6.1749785749609432E-2</v>
+        <v>1.4500000000000001E-2</v>
       </c>
       <c r="Q49">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.54040314349599206</v>
+        <v>1.46E-2</v>
       </c>
       <c r="R49">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.39614730741105397</v>
+        <v>1.47E-2</v>
       </c>
       <c r="S49">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.90161690277327378</v>
+        <v>1.4800000000000001E-2</v>
       </c>
       <c r="T49">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.57513361821908637</v>
+        <v>1.49E-2</v>
       </c>
       <c r="U49">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.168824441612625</v>
-      </c>
-    </row>
-    <row r="50" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="W49" s="7"/>
+      <c r="X49" s="7"/>
+      <c r="Y49" s="7"/>
+      <c r="Z49" s="7"/>
+      <c r="AA49" s="7"/>
+      <c r="AB49" s="7"/>
+    </row>
+    <row r="50" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
         <v>53</v>
       </c>
       <c r="B50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.1146621436989409</v>
+        <v>1.4E-2</v>
       </c>
       <c r="C50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.55001534938466456</v>
+        <v>1.4500000000000001E-2</v>
       </c>
       <c r="D50">
-        <f t="shared" ca="1" si="15"/>
-        <v>2.3136423202467782E-2</v>
+        <v>1.4666666666666672E-2</v>
       </c>
       <c r="E50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.94336117025919641</v>
+        <v>1.4833333333333329E-2</v>
       </c>
       <c r="F50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.95281489920284157</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="G50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.84108391750179468</v>
+        <v>1.52E-2</v>
       </c>
       <c r="H50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.41568614642178559</v>
+        <v>1.54E-2</v>
       </c>
       <c r="I50">
-        <f t="shared" ca="1" si="15"/>
-        <v>7.5178547249413752E-3</v>
+        <v>1.5599999999999999E-2</v>
       </c>
       <c r="J50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.19656972183605981</v>
+        <v>1.5800000000000002E-2</v>
       </c>
       <c r="K50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.66748175025529877</v>
+        <v>1.6E-2</v>
       </c>
       <c r="L50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.27827693107662876</v>
+        <v>1.61E-2</v>
       </c>
       <c r="M50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.81722333803023184</v>
+        <v>1.6199999999999999E-2</v>
       </c>
       <c r="N50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.7149933611610958</v>
+        <v>1.6299999999999999E-2</v>
       </c>
       <c r="O50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.90714047524822117</v>
+        <v>1.6400000000000001E-2</v>
       </c>
       <c r="P50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.6775229682415812</v>
+        <v>1.6500000000000001E-2</v>
       </c>
       <c r="Q50">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.26693236517595254</v>
+        <v>1.66E-2</v>
       </c>
       <c r="R50">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.38031240115159981</v>
+        <v>1.67E-2</v>
       </c>
       <c r="S50">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.24909809904355784</v>
+        <v>1.6799999999999999E-2</v>
       </c>
       <c r="T50">
-        <f t="shared" ca="1" si="16"/>
-        <v>9.56193530102315E-2</v>
+        <v>1.6899999999999998E-2</v>
       </c>
       <c r="U50">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.30945106324905824</v>
-      </c>
-    </row>
-    <row r="51" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+        <v>1.7000000000000001E-2</v>
+      </c>
+      <c r="W50" s="7"/>
+      <c r="X50" s="7"/>
+      <c r="Y50" s="7"/>
+      <c r="Z50" s="7"/>
+      <c r="AA50" s="7"/>
+      <c r="AB50" s="7"/>
+    </row>
+    <row r="51" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
         <v>54</v>
       </c>
       <c r="B51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.35741480167658213</v>
+        <v>1.6E-2</v>
       </c>
       <c r="C51">
-        <f t="shared" ca="1" si="15"/>
-        <v>1.9036224580679328E-2</v>
+        <v>1.6500000000000001E-2</v>
       </c>
       <c r="D51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.22419873414011027</v>
+        <v>1.666666666666667E-2</v>
       </c>
       <c r="E51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.48553231140032216</v>
+        <v>1.6833333333333329E-2</v>
       </c>
       <c r="F51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.46961604796492284</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="G51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.11523427327605629</v>
+        <v>1.72E-2</v>
       </c>
       <c r="H51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.35291075674254624</v>
+        <v>1.7399999999999999E-2</v>
       </c>
       <c r="I51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.65266088113824805</v>
+        <v>1.7600000000000001E-2</v>
       </c>
       <c r="J51">
-        <f t="shared" ca="1" si="15"/>
-        <v>8.5936979363917976E-2</v>
+        <v>1.78E-2</v>
       </c>
       <c r="K51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.80359335736910475</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="L51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.55358728290000803</v>
+        <v>1.8100000000000002E-2</v>
       </c>
       <c r="M51">
-        <f t="shared" ca="1" si="15"/>
-        <v>1.2239702437443212E-3</v>
+        <v>1.8200000000000001E-2</v>
       </c>
       <c r="N51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.29779659955661375</v>
+        <v>1.83E-2</v>
       </c>
       <c r="O51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.8776412456781888</v>
+        <v>1.84E-2</v>
       </c>
       <c r="P51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.82163221467805925</v>
+        <v>1.8499999999999999E-2</v>
       </c>
       <c r="Q51">
-        <f t="shared" ca="1" si="15"/>
-        <v>0.98053884439076777</v>
+        <v>1.8599999999999998E-2</v>
       </c>
       <c r="R51">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.64550818962162115</v>
+        <v>1.8700000000000001E-2</v>
       </c>
       <c r="S51">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.10808415852876641</v>
+        <v>1.8800000000000001E-2</v>
       </c>
       <c r="T51">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.86322220360281954</v>
+        <v>1.89E-2</v>
       </c>
       <c r="U51">
-        <f t="shared" ca="1" si="16"/>
-        <v>0.90397349298902219</v>
-      </c>
-    </row>
-    <row r="52" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+        <v>1.9E-2</v>
+      </c>
+      <c r="X51" s="7"/>
+      <c r="Y51" s="7"/>
+      <c r="Z51" s="7"/>
+      <c r="AA51" s="7"/>
+      <c r="AB51" s="7"/>
+    </row>
+    <row r="52" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
         <v>55</v>
       </c>
       <c r="B52" s="4">
-        <v>0</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="C52" s="4">
-        <v>0</v>
+        <v>1.8499999999999999E-2</v>
       </c>
       <c r="D52" s="4">
-        <v>0</v>
+        <v>1.8666666666666672E-2</v>
       </c>
       <c r="E52" s="4">
-        <v>0</v>
+        <v>1.8833333333333327E-2</v>
       </c>
       <c r="F52" s="4">
-        <v>0</v>
+        <v>1.9E-2</v>
       </c>
       <c r="G52" s="4">
-        <v>0</v>
+        <v>1.9199999999999998E-2</v>
       </c>
       <c r="H52" s="4">
-        <v>0</v>
+        <v>1.9400000000000001E-2</v>
       </c>
       <c r="I52" s="4">
-        <v>0</v>
+        <v>1.9599999999999999E-2</v>
       </c>
       <c r="J52" s="4">
-        <v>0</v>
+        <v>1.9800000000000002E-2</v>
       </c>
       <c r="K52" s="4">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="L52" s="4">
-        <v>0</v>
+        <v>2.01E-2</v>
       </c>
       <c r="M52" s="4">
-        <v>0</v>
+        <v>2.0199999999999999E-2</v>
       </c>
       <c r="N52" s="4">
-        <v>0</v>
+        <v>2.0299999999999999E-2</v>
       </c>
       <c r="O52" s="4">
-        <v>0</v>
+        <v>2.0400000000000001E-2</v>
       </c>
       <c r="P52" s="4">
-        <v>0</v>
+        <v>2.0500000000000001E-2</v>
       </c>
       <c r="Q52" s="4">
-        <v>0</v>
+        <v>2.06E-2</v>
       </c>
       <c r="R52" s="4">
-        <v>0</v>
+        <v>2.07E-2</v>
       </c>
       <c r="S52" s="4">
-        <v>0</v>
+        <v>2.0799999999999999E-2</v>
       </c>
       <c r="T52" s="4">
-        <v>0</v>
+        <v>2.0899999999999998E-2</v>
       </c>
       <c r="U52" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="X52" s="7"/>
+      <c r="Y52" s="7"/>
+      <c r="Z52" s="7"/>
+      <c r="AA52" s="7"/>
+      <c r="AB52" s="7"/>
+    </row>
+    <row r="53" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
         <v>56</v>
       </c>
       <c r="B53" s="4">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="C53" s="4">
-        <v>0</v>
+        <v>2.0500000000000001E-2</v>
       </c>
       <c r="D53" s="4">
-        <v>0</v>
+        <v>2.066666666666667E-2</v>
       </c>
       <c r="E53" s="4">
-        <v>0</v>
+        <v>2.0833333333333329E-2</v>
       </c>
       <c r="F53" s="4">
-        <v>0</v>
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="G53" s="4">
-        <v>0</v>
+        <v>2.12E-2</v>
       </c>
       <c r="H53" s="4">
-        <v>0</v>
+        <v>2.1399999999999999E-2</v>
       </c>
       <c r="I53" s="4">
-        <v>0</v>
+        <v>2.1600000000000001E-2</v>
       </c>
       <c r="J53" s="4">
-        <v>0</v>
+        <v>2.18E-2</v>
       </c>
       <c r="K53" s="4">
-        <v>0</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="L53" s="4">
-        <v>0</v>
+        <v>2.2100000000000002E-2</v>
       </c>
       <c r="M53" s="4">
-        <v>0</v>
+        <v>2.2200000000000001E-2</v>
       </c>
       <c r="N53" s="4">
-        <v>0</v>
+        <v>2.23E-2</v>
       </c>
       <c r="O53" s="4">
-        <v>0</v>
+        <v>2.24E-2</v>
       </c>
       <c r="P53" s="4">
-        <v>0</v>
+        <v>2.2499999999999999E-2</v>
       </c>
       <c r="Q53" s="4">
-        <v>0</v>
+        <v>2.2599999999999999E-2</v>
       </c>
       <c r="R53" s="4">
-        <v>0</v>
+        <v>2.2700000000000001E-2</v>
       </c>
       <c r="S53" s="4">
-        <v>0</v>
+        <v>2.2800000000000001E-2</v>
       </c>
       <c r="T53" s="4">
-        <v>0</v>
+        <v>2.29E-2</v>
       </c>
       <c r="U53" s="4">
-        <v>0</v>
-      </c>
+        <v>2.3E-2</v>
+      </c>
+      <c r="X53" s="7"/>
+      <c r="Y53" s="7"/>
+      <c r="Z53" s="7"/>
+      <c r="AA53" s="7"/>
+      <c r="AB53" s="7"/>
+    </row>
+    <row r="54" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="X54" s="7"/>
+      <c r="Y54" s="7"/>
+      <c r="Z54" s="7"/>
+      <c r="AA54" s="7"/>
+      <c r="AB54" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
SII Review Tool: Adding a low-interest rate scenario.
</commit_message>
<xml_diff>
--- a/inputs.xlsx
+++ b/inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\d-fine\Projects\SII Review Tool\SII Review Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8E182A-8F93-4563-A0BE-F5AE984E7498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5965FBC8-9A67-4CA9-B322-8C695AD36BED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="zero_rates_alt" sheetId="1" r:id="rId1"/>
@@ -2921,7 +2921,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B12">
         <v>11</v>
@@ -2943,7 +2943,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B14">
         <v>13</v>
@@ -2954,7 +2954,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15">
         <v>14</v>
@@ -2976,7 +2976,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17">
         <v>16</v>
@@ -2987,7 +2987,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18">
         <v>17</v>
@@ -2998,7 +2998,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B19">
         <v>18</v>
@@ -3009,7 +3009,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20">
         <v>19</v>

</xml_diff>

<commit_message>
SII Review Tool: Adding externally computed va spread values.
</commit_message>
<xml_diff>
--- a/inputs.xlsx
+++ b/inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\d-fine\Projects\SII Review Tool\SII Review Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5965FBC8-9A67-4CA9-B322-8C695AD36BED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB54F301-C41E-4029-8936-BA98FE0D7196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43200" yWindow="0" windowWidth="14400" windowHeight="15600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="zero_rates_alt" sheetId="1" r:id="rId1"/>
@@ -6004,7 +6004,7 @@
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B23">
@@ -6134,7 +6134,7 @@
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B25" s="6">
@@ -6199,7 +6199,7 @@
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B26">
@@ -6329,7 +6329,7 @@
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B28" s="6">
@@ -6394,7 +6394,7 @@
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B29" s="6">
@@ -6459,7 +6459,7 @@
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B30">
@@ -6654,7 +6654,7 @@
       </c>
     </row>
     <row r="33" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B33">
@@ -6719,7 +6719,7 @@
       </c>
     </row>
     <row r="34" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B34">
@@ -6784,7 +6784,7 @@
       </c>
     </row>
     <row r="35" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B35" s="6">
@@ -6849,7 +6849,7 @@
       </c>
     </row>
     <row r="36" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A36" s="3" t="s">
+      <c r="A36" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B36" s="6">
@@ -6979,7 +6979,7 @@
       </c>
     </row>
     <row r="38" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A38" s="3" t="s">
+      <c r="A38" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B38">
@@ -7044,7 +7044,7 @@
       </c>
     </row>
     <row r="39" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A39" s="3" t="s">
+      <c r="A39" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B39">
@@ -7109,7 +7109,7 @@
       </c>
     </row>
     <row r="40" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B40">
@@ -7174,7 +7174,7 @@
       </c>
     </row>
     <row r="41" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A41" s="3" t="s">
+      <c r="A41" s="2" t="s">
         <v>44</v>
       </c>
       <c r="B41">
@@ -7245,7 +7245,7 @@
       <c r="AB41" s="5"/>
     </row>
     <row r="42" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="2" t="s">
         <v>45</v>
       </c>
       <c r="B42">
@@ -7316,7 +7316,7 @@
       <c r="AB42" s="5"/>
     </row>
     <row r="43" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B43">
@@ -7387,7 +7387,7 @@
       <c r="AB43" s="5"/>
     </row>
     <row r="44" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A44" s="3" t="s">
+      <c r="A44" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B44">
@@ -7600,7 +7600,7 @@
       <c r="AB46" s="5"/>
     </row>
     <row r="47" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="2" t="s">
         <v>50</v>
       </c>
       <c r="B47">
@@ -7666,7 +7666,7 @@
       <c r="W47" s="5"/>
     </row>
     <row r="48" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A48" s="3" t="s">
+      <c r="A48" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B48">
@@ -7737,7 +7737,7 @@
       <c r="AB48" s="5"/>
     </row>
     <row r="49" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B49">
@@ -7808,7 +7808,7 @@
       <c r="AB49" s="5"/>
     </row>
     <row r="50" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A50" s="3" t="s">
+      <c r="A50" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B50">
@@ -7879,7 +7879,7 @@
       <c r="AB50" s="5"/>
     </row>
     <row r="51" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="2" t="s">
         <v>54</v>
       </c>
       <c r="B51">

</xml_diff>